<commit_message>
chore(data): sync latest portfolio snapshot
</commit_message>
<xml_diff>
--- a/assets.xlsx
+++ b/assets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Final_Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chart" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Exec" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet name="Daily" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet name="Dashboard" sheetId="6" state="hidden" r:id="rId6"/>
-    <sheet name="Hidden_Logic" sheetId="7" state="hidden" r:id="rId7"/>
-    <sheet name="Holdings" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final_Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exec" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hidden_Logic" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holdings" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -807,14 +807,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr lvl="0">
               <a:defRPr sz="1400" b="1">
                 <a:solidFill>
@@ -861,7 +861,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln cmpd="sng">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cmpd="sng">
               <a:solidFill>
                 <a:srgbClr val="0A84FF"/>
               </a:solidFill>
@@ -871,7 +871,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -902,9 +902,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr lvl="0">
                   <a:defRPr b="0">
                     <a:solidFill>
@@ -931,14 +931,14 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:ln>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr lvl="0">
               <a:defRPr b="0">
                 <a:solidFill>
@@ -965,7 +965,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="B7B7B7"/>
               </a:solidFill>
@@ -975,7 +975,7 @@
         </majorGridlines>
         <minorGridlines>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="CCCCCC"/>
               </a:solidFill>
@@ -986,9 +986,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr lvl="0">
                   <a:defRPr b="0">
                     <a:solidFill>
@@ -1016,14 +1016,14 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr lvl="0">
               <a:defRPr b="0">
                 <a:solidFill>
@@ -1047,14 +1047,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr lvl="0">
               <a:defRPr b="0">
                 <a:solidFill>
@@ -1091,7 +1091,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln cmpd="sng">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cmpd="sng">
               <a:solidFill>
                 <a:srgbClr val="4285F4"/>
               </a:solidFill>
@@ -1101,7 +1101,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1132,9 +1132,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr lvl="0">
                   <a:defRPr b="0">
                     <a:solidFill>
@@ -1161,14 +1161,14 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:ln>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr lvl="0">
               <a:defRPr b="0">
                 <a:solidFill>
@@ -1195,7 +1195,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="B7B7B7"/>
               </a:solidFill>
@@ -1205,7 +1205,7 @@
         </majorGridlines>
         <minorGridlines>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="CCCCCC"/>
               </a:solidFill>
@@ -1216,9 +1216,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr lvl="0">
                   <a:defRPr b="0">
                     <a:solidFill>
@@ -1246,14 +1246,14 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr lvl="0">
               <a:defRPr b="0">
                 <a:solidFill>
@@ -1274,9 +1274,9 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr lvl="0">
             <a:defRPr b="0">
               <a:solidFill>
@@ -1298,14 +1298,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr lvl="0">
               <a:defRPr sz="1600" b="1">
                 <a:solidFill>
@@ -1341,7 +1341,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln cmpd="sng">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cmpd="sng">
               <a:solidFill>
                 <a:srgbClr val="236BE5"/>
               </a:solidFill>
@@ -1351,7 +1351,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1378,7 +1378,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln cmpd="sng">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cmpd="sng">
               <a:solidFill>
                 <a:srgbClr val="DB332D"/>
               </a:solidFill>
@@ -1388,7 +1388,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1419,9 +1419,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr lvl="0">
                   <a:defRPr b="0">
                     <a:solidFill>
@@ -1448,14 +1448,14 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
-          <a:ln>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr lvl="0">
               <a:defRPr b="0">
                 <a:solidFill>
@@ -1481,7 +1481,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="B7B7B7"/>
               </a:solidFill>
@@ -1491,7 +1491,7 @@
         </majorGridlines>
         <minorGridlines>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="CCCCCC"/>
               </a:solidFill>
@@ -1502,9 +1502,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr lvl="0">
                   <a:defRPr b="0">
                     <a:solidFill>
@@ -1532,14 +1532,14 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr lvl="0">
               <a:defRPr b="0">
                 <a:solidFill>
@@ -1560,9 +1560,9 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr lvl="0">
             <a:defRPr b="0">
               <a:solidFill>
@@ -1581,10 +1581,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:prstDash val="solid"/>
     </a:ln>
   </spPr>
@@ -1611,7 +1611,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1626,9 +1626,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1638,7 +1638,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -1653,9 +1653,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1675,9 +1675,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -10005,8 +10005,14 @@
       <c r="Z190" s="51" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="67" t="n"/>
-      <c r="B191" s="64" t="n"/>
+      <c r="A191" s="67" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B191" s="64" t="n">
+        <v>1.2689</v>
+      </c>
       <c r="C191" s="64" t="n"/>
       <c r="D191" s="64" t="n"/>
       <c r="E191" s="67" t="n"/>
@@ -10033,8 +10039,14 @@
       <c r="Z191" s="51" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="67" t="n"/>
-      <c r="B192" s="64" t="n"/>
+      <c r="A192" s="67" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B192" s="64" t="n">
+        <v>1.2689</v>
+      </c>
       <c r="C192" s="64" t="n"/>
       <c r="D192" s="64" t="n"/>
       <c r="E192" s="67" t="n"/>
@@ -10061,8 +10073,14 @@
       <c r="Z192" s="51" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="67" t="n"/>
-      <c r="B193" s="64" t="n"/>
+      <c r="A193" s="67" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B193" s="64" t="n">
+        <v>1.2588</v>
+      </c>
       <c r="C193" s="64" t="n"/>
       <c r="D193" s="64" t="n"/>
       <c r="E193" s="67" t="n"/>
@@ -10089,8 +10107,14 @@
       <c r="Z193" s="51" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="67" t="n"/>
-      <c r="B194" s="64" t="n"/>
+      <c r="A194" s="67" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="B194" s="64" t="n">
+        <v>1.2663</v>
+      </c>
       <c r="C194" s="64" t="n"/>
       <c r="D194" s="64" t="n"/>
       <c r="E194" s="67" t="n"/>
@@ -32736,7 +32760,7 @@
         </is>
       </c>
       <c r="B2" s="77" t="n">
-        <v>46082.74882633071</v>
+        <v>46086.75502439712</v>
       </c>
       <c r="C2" s="86" t="inlineStr">
         <is>
@@ -32790,7 +32814,7 @@
         </is>
       </c>
       <c r="H3" s="122" t="n">
-        <v>46082.74882633071</v>
+        <v>46086.75502439712</v>
       </c>
       <c r="I3" s="99" t="n"/>
       <c r="J3" s="99" t="n"/>
@@ -46665,13 +46689,31 @@
       <c r="T190" s="99" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="99" t="n"/>
-      <c r="B191" s="117" t="n"/>
-      <c r="C191" s="117" t="n"/>
-      <c r="D191" s="117" t="n"/>
-      <c r="E191" s="117" t="n"/>
-      <c r="F191" s="91" t="n"/>
-      <c r="G191" s="117" t="n"/>
+      <c r="A191" s="99" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B191" s="117" t="n">
+        <v>571.73</v>
+      </c>
+      <c r="C191" s="117" t="n">
+        <v>1510.08</v>
+      </c>
+      <c r="D191" s="117" t="n">
+        <v>3199.7</v>
+      </c>
+      <c r="E191" s="117" t="n">
+        <v>5281.51</v>
+      </c>
+      <c r="F191" s="91" t="n">
+        <v>1.2689</v>
+      </c>
+      <c r="G191" s="123" t="inlineStr">
+        <is>
+          <t>carry</t>
+        </is>
+      </c>
       <c r="H191" s="117" t="n"/>
       <c r="I191" s="99" t="n"/>
       <c r="J191" s="99" t="n"/>
@@ -46687,13 +46729,31 @@
       <c r="T191" s="99" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="99" t="n"/>
-      <c r="B192" s="117" t="n"/>
-      <c r="C192" s="117" t="n"/>
-      <c r="D192" s="117" t="n"/>
-      <c r="E192" s="117" t="n"/>
-      <c r="F192" s="91" t="n"/>
-      <c r="G192" s="117" t="n"/>
+      <c r="A192" s="99" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B192" s="117" t="n">
+        <v>571.73</v>
+      </c>
+      <c r="C192" s="117" t="n">
+        <v>1510.08</v>
+      </c>
+      <c r="D192" s="117" t="n">
+        <v>3199.7</v>
+      </c>
+      <c r="E192" s="117" t="n">
+        <v>5281.51</v>
+      </c>
+      <c r="F192" s="91" t="n">
+        <v>1.2689</v>
+      </c>
+      <c r="G192" s="123" t="inlineStr">
+        <is>
+          <t>carry</t>
+        </is>
+      </c>
       <c r="H192" s="117" t="n"/>
       <c r="I192" s="99" t="n"/>
       <c r="J192" s="99" t="n"/>
@@ -46709,13 +46769,31 @@
       <c r="T192" s="99" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="99" t="n"/>
-      <c r="B193" s="117" t="n"/>
-      <c r="C193" s="117" t="n"/>
-      <c r="D193" s="117" t="n"/>
-      <c r="E193" s="117" t="n"/>
-      <c r="F193" s="91" t="n"/>
-      <c r="G193" s="117" t="n"/>
+      <c r="A193" s="99" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B193" s="117" t="n">
+        <v>571.73</v>
+      </c>
+      <c r="C193" s="117" t="n">
+        <v>1491.75</v>
+      </c>
+      <c r="D193" s="117" t="n">
+        <v>3175.92</v>
+      </c>
+      <c r="E193" s="117" t="n">
+        <v>5239.4</v>
+      </c>
+      <c r="F193" s="91" t="n">
+        <v>1.2588</v>
+      </c>
+      <c r="G193" s="123" t="inlineStr">
+        <is>
+          <t>broker-sync</t>
+        </is>
+      </c>
       <c r="H193" s="117" t="n"/>
       <c r="I193" s="99" t="n"/>
       <c r="J193" s="99" t="n"/>
@@ -46731,13 +46809,31 @@
       <c r="T193" s="99" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="99" t="n"/>
-      <c r="B194" s="117" t="n"/>
-      <c r="C194" s="117" t="n"/>
-      <c r="D194" s="117" t="n"/>
-      <c r="E194" s="117" t="n"/>
-      <c r="F194" s="91" t="n"/>
-      <c r="G194" s="117" t="n"/>
+      <c r="A194" s="99" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="B194" s="117" t="n">
+        <v>571.73</v>
+      </c>
+      <c r="C194" s="117" t="n">
+        <v>1488.33</v>
+      </c>
+      <c r="D194" s="117" t="n">
+        <v>3210.55</v>
+      </c>
+      <c r="E194" s="117" t="n">
+        <v>5270.61</v>
+      </c>
+      <c r="F194" s="91" t="n">
+        <v>1.2663</v>
+      </c>
+      <c r="G194" s="123" t="inlineStr">
+        <is>
+          <t>broker-sync</t>
+        </is>
+      </c>
       <c r="H194" s="117" t="n"/>
       <c r="I194" s="99" t="n"/>
       <c r="J194" s="99" t="n"/>
@@ -63159,7 +63255,7 @@
     </row>
     <row r="2">
       <c r="A2" s="121" t="n">
-        <v>46082.74882633071</v>
+        <v>46086.75502439712</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
@@ -63180,15 +63276,15 @@
         <v>0.734</v>
       </c>
       <c r="F2" s="0" t="n">
-        <v>177.1900024414062</v>
+        <v>183.0399932861328</v>
       </c>
       <c r="G2" s="0" t="n">
-        <v>130.0574617919922</v>
+        <v>134.3513550720215</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="121" t="n">
-        <v>46082.74882633071</v>
+        <v>46086.75502439712</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
@@ -63209,15 +63305,15 @@
         <v>15.1446</v>
       </c>
       <c r="F3" s="0" t="n">
-        <v>100.6399993896484</v>
+        <v>100.4000015258789</v>
       </c>
       <c r="G3" s="0" t="n">
-        <v>1524.15253475647</v>
+        <v>1520.517863108826</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="121" t="n">
-        <v>46082.74882633071</v>
+        <v>46086.75502439712</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
@@ -63238,15 +63334,15 @@
         <v>1.2254</v>
       </c>
       <c r="F4" s="0" t="n">
-        <v>402.510009765625</v>
+        <v>405.9400024414062</v>
       </c>
       <c r="G4" s="0" t="n">
-        <v>493.2357659667969</v>
+        <v>497.4388789916993</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="121" t="n">
-        <v>46082.74882633071</v>
+        <v>46086.75502439712</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
@@ -63267,15 +63363,15 @@
         <v>1.7327</v>
       </c>
       <c r="F5" s="0" t="n">
-        <v>607.2899780273438</v>
+        <v>610.75</v>
       </c>
       <c r="G5" s="0" t="n">
-        <v>1052.251344927978</v>
+        <v>1058.246525</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="121" t="n">
-        <v>46082.74882633071</v>
+        <v>46086.75502439712</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
@@ -63304,7 +63400,7 @@
     </row>
     <row r="7">
       <c r="A7" s="121" t="n">
-        <v>46082.74882633071</v>
+        <v>46086.75502439712</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
@@ -63325,10 +63421,10 @@
         <v>0.28775</v>
       </c>
       <c r="F7" s="0" t="n">
-        <v>5247.89990234375</v>
+        <v>5172.2998046875</v>
       </c>
       <c r="G7" s="0" t="n">
-        <v>1510.083196899414</v>
+        <v>1488.329268798828</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: add failure alerts and stable script entrypoint for cron
</commit_message>
<xml_diff>
--- a/assets.xlsx
+++ b/assets.xlsx
@@ -10113,7 +10113,7 @@
         </is>
       </c>
       <c r="B194" s="64" t="n">
-        <v>1.2663</v>
+        <v>1.2656</v>
       </c>
       <c r="C194" s="64" t="n"/>
       <c r="D194" s="64" t="n"/>
@@ -32760,7 +32760,7 @@
         </is>
       </c>
       <c r="B2" s="77" t="n">
-        <v>46086.75502439712</v>
+        <v>46086.76015296084</v>
       </c>
       <c r="C2" s="86" t="inlineStr">
         <is>
@@ -32814,7 +32814,7 @@
         </is>
       </c>
       <c r="H3" s="122" t="n">
-        <v>46086.75502439712</v>
+        <v>46086.76015296084</v>
       </c>
       <c r="I3" s="99" t="n"/>
       <c r="J3" s="99" t="n"/>
@@ -46818,16 +46818,16 @@
         <v>571.73</v>
       </c>
       <c r="C194" s="117" t="n">
-        <v>1488.33</v>
+        <v>1485.31</v>
       </c>
       <c r="D194" s="117" t="n">
         <v>3210.55</v>
       </c>
       <c r="E194" s="117" t="n">
-        <v>5270.61</v>
+        <v>5267.59</v>
       </c>
       <c r="F194" s="91" t="n">
-        <v>1.2663</v>
+        <v>1.2656</v>
       </c>
       <c r="G194" s="123" t="inlineStr">
         <is>
@@ -63255,7 +63255,7 @@
     </row>
     <row r="2">
       <c r="A2" s="121" t="n">
-        <v>46086.75502439712</v>
+        <v>46086.76015296084</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
@@ -63284,7 +63284,7 @@
     </row>
     <row r="3">
       <c r="A3" s="121" t="n">
-        <v>46086.75502439712</v>
+        <v>46086.76015296084</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
@@ -63313,7 +63313,7 @@
     </row>
     <row r="4">
       <c r="A4" s="121" t="n">
-        <v>46086.75502439712</v>
+        <v>46086.76015296084</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
@@ -63342,7 +63342,7 @@
     </row>
     <row r="5">
       <c r="A5" s="121" t="n">
-        <v>46086.75502439712</v>
+        <v>46086.76015296084</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
@@ -63371,7 +63371,7 @@
     </row>
     <row r="6">
       <c r="A6" s="121" t="n">
-        <v>46086.75502439712</v>
+        <v>46086.76015296084</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
@@ -63400,7 +63400,7 @@
     </row>
     <row r="7">
       <c r="A7" s="121" t="n">
-        <v>46086.75502439712</v>
+        <v>46086.76015296084</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
@@ -63421,10 +63421,10 @@
         <v>0.28775</v>
       </c>
       <c r="F7" s="0" t="n">
-        <v>5172.2998046875</v>
+        <v>5161.7998046875</v>
       </c>
       <c r="G7" s="0" t="n">
-        <v>1488.329268798828</v>
+        <v>1485.307893798828</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): sync portfolio data 2026-03-05 18:15:24 CST
</commit_message>
<xml_diff>
--- a/assets.xlsx
+++ b/assets.xlsx
@@ -32760,7 +32760,7 @@
         </is>
       </c>
       <c r="B2" s="77" t="n">
-        <v>46086.76015296084</v>
+        <v>46086.76059091686</v>
       </c>
       <c r="C2" s="86" t="inlineStr">
         <is>
@@ -32814,7 +32814,7 @@
         </is>
       </c>
       <c r="H3" s="122" t="n">
-        <v>46086.76015296084</v>
+        <v>46086.76059091686</v>
       </c>
       <c r="I3" s="99" t="n"/>
       <c r="J3" s="99" t="n"/>
@@ -46818,13 +46818,13 @@
         <v>571.73</v>
       </c>
       <c r="C194" s="117" t="n">
-        <v>1485.31</v>
+        <v>1485.42</v>
       </c>
       <c r="D194" s="117" t="n">
         <v>3210.55</v>
       </c>
       <c r="E194" s="117" t="n">
-        <v>5267.59</v>
+        <v>5267.71</v>
       </c>
       <c r="F194" s="91" t="n">
         <v>1.2656</v>
@@ -63255,7 +63255,7 @@
     </row>
     <row r="2">
       <c r="A2" s="121" t="n">
-        <v>46086.76015296084</v>
+        <v>46086.76059091686</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
@@ -63284,7 +63284,7 @@
     </row>
     <row r="3">
       <c r="A3" s="121" t="n">
-        <v>46086.76015296084</v>
+        <v>46086.76059091686</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
@@ -63313,7 +63313,7 @@
     </row>
     <row r="4">
       <c r="A4" s="121" t="n">
-        <v>46086.76015296084</v>
+        <v>46086.76059091686</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
@@ -63342,7 +63342,7 @@
     </row>
     <row r="5">
       <c r="A5" s="121" t="n">
-        <v>46086.76015296084</v>
+        <v>46086.76059091686</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
@@ -63371,7 +63371,7 @@
     </row>
     <row r="6">
       <c r="A6" s="121" t="n">
-        <v>46086.76015296084</v>
+        <v>46086.76059091686</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
@@ -63400,7 +63400,7 @@
     </row>
     <row r="7">
       <c r="A7" s="121" t="n">
-        <v>46086.76015296084</v>
+        <v>46086.76059091686</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
@@ -63421,10 +63421,10 @@
         <v>0.28775</v>
       </c>
       <c r="F7" s="0" t="n">
-        <v>5161.7998046875</v>
+        <v>5162.2001953125</v>
       </c>
       <c r="G7" s="0" t="n">
-        <v>1485.307893798828</v>
+        <v>1485.423106201172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): sync gold holding to latest cny value
</commit_message>
<xml_diff>
--- a/assets.xlsx
+++ b/assets.xlsx
@@ -10141,8 +10141,14 @@
       <c r="Z194" s="51" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="67" t="n"/>
-      <c r="B195" s="64" t="n"/>
+      <c r="A195" s="67" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B195" s="64" t="n">
+        <v>1.3408</v>
+      </c>
       <c r="C195" s="64" t="n"/>
       <c r="D195" s="64" t="n"/>
       <c r="E195" s="67" t="n"/>
@@ -32760,7 +32766,7 @@
         </is>
       </c>
       <c r="B2" s="77" t="n">
-        <v>46086.76059091686</v>
+        <v>46087.70724480331</v>
       </c>
       <c r="C2" s="86" t="inlineStr">
         <is>
@@ -32814,7 +32820,7 @@
         </is>
       </c>
       <c r="H3" s="122" t="n">
-        <v>46086.76059091686</v>
+        <v>46087.70724480331</v>
       </c>
       <c r="I3" s="99" t="n"/>
       <c r="J3" s="99" t="n"/>
@@ -46818,13 +46824,13 @@
         <v>571.73</v>
       </c>
       <c r="C194" s="117" t="n">
-        <v>1485.42</v>
+        <v>1485.25</v>
       </c>
       <c r="D194" s="117" t="n">
         <v>3210.55</v>
       </c>
       <c r="E194" s="117" t="n">
-        <v>5267.71</v>
+        <v>5267.54</v>
       </c>
       <c r="F194" s="91" t="n">
         <v>1.2656</v>
@@ -46849,13 +46855,31 @@
       <c r="T194" s="99" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="99" t="n"/>
-      <c r="B195" s="117" t="n"/>
-      <c r="C195" s="117" t="n"/>
-      <c r="D195" s="117" t="n"/>
-      <c r="E195" s="117" t="n"/>
-      <c r="F195" s="91" t="n"/>
-      <c r="G195" s="117" t="n"/>
+      <c r="A195" s="99" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B195" s="117" t="n">
+        <v>571.73</v>
+      </c>
+      <c r="C195" s="117" t="n">
+        <v>1801.49</v>
+      </c>
+      <c r="D195" s="117" t="n">
+        <v>3207.26</v>
+      </c>
+      <c r="E195" s="117" t="n">
+        <v>5580.48</v>
+      </c>
+      <c r="F195" s="91" t="n">
+        <v>1.3408</v>
+      </c>
+      <c r="G195" s="123" t="inlineStr">
+        <is>
+          <t>broker-sync</t>
+        </is>
+      </c>
       <c r="H195" s="117" t="n"/>
       <c r="I195" s="99" t="n"/>
       <c r="J195" s="99" t="n"/>
@@ -63255,7 +63279,7 @@
     </row>
     <row r="2">
       <c r="A2" s="121" t="n">
-        <v>46086.76059091686</v>
+        <v>46087.70724480331</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
@@ -63276,15 +63300,15 @@
         <v>0.734</v>
       </c>
       <c r="F2" s="0" t="n">
-        <v>183.0399932861328</v>
+        <v>183.3399963378906</v>
       </c>
       <c r="G2" s="0" t="n">
-        <v>134.3513550720215</v>
+        <v>134.5715573120117</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="121" t="n">
-        <v>46086.76059091686</v>
+        <v>46087.70724480331</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
@@ -63305,15 +63329,15 @@
         <v>15.1446</v>
       </c>
       <c r="F3" s="0" t="n">
-        <v>100.4000015258789</v>
+        <v>100.4100036621094</v>
       </c>
       <c r="G3" s="0" t="n">
-        <v>1520.517863108826</v>
+        <v>1520.669341461182</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="121" t="n">
-        <v>46086.76059091686</v>
+        <v>46087.70724480331</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
@@ -63334,15 +63358,15 @@
         <v>1.2254</v>
       </c>
       <c r="F4" s="0" t="n">
-        <v>405.9400024414062</v>
+        <v>405.5499877929688</v>
       </c>
       <c r="G4" s="0" t="n">
-        <v>497.4388789916993</v>
+        <v>496.960955041504</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="121" t="n">
-        <v>46086.76059091686</v>
+        <v>46087.70724480331</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
@@ -63363,15 +63387,15 @@
         <v>1.7327</v>
       </c>
       <c r="F5" s="0" t="n">
-        <v>610.75</v>
+        <v>608.9099731445312</v>
       </c>
       <c r="G5" s="0" t="n">
-        <v>1058.246525</v>
+        <v>1055.058310467529</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="121" t="n">
-        <v>46086.76059091686</v>
+        <v>46087.70724480331</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
@@ -63400,7 +63424,7 @@
     </row>
     <row r="7">
       <c r="A7" s="121" t="n">
-        <v>46086.76059091686</v>
+        <v>46087.70724480331</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
@@ -63418,13 +63442,13 @@
         </is>
       </c>
       <c r="E7" s="0" t="n">
-        <v>0.28775</v>
+        <v>0.351785122969631</v>
       </c>
       <c r="F7" s="0" t="n">
-        <v>5162.2001953125</v>
+        <v>5121</v>
       </c>
       <c r="G7" s="0" t="n">
-        <v>1485.423106201172</v>
+        <v>1801.49161472748</v>
       </c>
     </row>
   </sheetData>

</xml_diff>